<commit_message>
feat(workbook): caixa final, bloqueado e retiradas nas entradas do fechamento
- Caixa final (saldo do extrato) informado no fechamento: a diferença para o
  caixa calculado vira ajuste do mês (coluna AO da BASE), somado ao caixa
  acumulado da aba Receita; os meses seguintes partem do caixa informado.
- Bloqueado passa a ser só informado no fechamento (antes: soma atual dos
  limites dos cartões, igual em todos os meses).
- Saldo anterior do caixa inclui dez/(ano-3), que ficava fora do modelo.
- Janela "Entradas do fechamento" com seções de redes sociais, caixa (com o
  valor calculado e o ajuste), sócios/FOPAG (retiradas e saldo do mês, só
  leitura) e parâmetros do ano.
- BASE grava as células de cada linha em ordem de coluna.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X7r1acLXPYnBHUwEgBcPmn
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v1.xlsx
+++ b/public/workbook_fechamento_v1.xlsx
@@ -27449,40 +27449,40 @@
         <v>98</v>
       </c>
       <c r="C3" s="1052">
-        <f>IF(BASE!$B$3=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:C4),"")</f>
+        <f>IF(BASE!$B$3=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:C4)+SUM(BASE!$AO$3:$AO$3)/1000,"")</f>
       </c>
       <c r="D3" s="1052">
-        <f>IF(BASE!$B$4=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:D4),"")</f>
+        <f>IF(BASE!$B$4=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:D4)+SUM(BASE!$AO$3:$AO$4)/1000,"")</f>
       </c>
       <c r="E3" s="1052">
-        <f>IF(BASE!$B$5=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:E4),"")</f>
+        <f>IF(BASE!$B$5=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:E4)+SUM(BASE!$AO$3:$AO$5)/1000,"")</f>
       </c>
       <c r="F3" s="1052">
-        <f>IF(BASE!$B$6=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:F4),"")</f>
+        <f>IF(BASE!$B$6=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:F4)+SUM(BASE!$AO$3:$AO$6)/1000,"")</f>
       </c>
       <c r="G3" s="1052">
-        <f>IF(BASE!$B$7=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:G4),"")</f>
+        <f>IF(BASE!$B$7=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:G4)+SUM(BASE!$AO$3:$AO$7)/1000,"")</f>
       </c>
       <c r="H3" s="1052">
-        <f>IF(BASE!$B$8=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:H4),"")</f>
+        <f>IF(BASE!$B$8=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:H4)+SUM(BASE!$AO$3:$AO$8)/1000,"")</f>
       </c>
       <c r="I3" s="1052">
-        <f>IF(BASE!$B$9=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:I4),"")</f>
+        <f>IF(BASE!$B$9=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:I4)+SUM(BASE!$AO$3:$AO$9)/1000,"")</f>
       </c>
       <c r="J3" s="1052">
-        <f>IF(BASE!$B$10=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:J4),"")</f>
+        <f>IF(BASE!$B$10=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:J4)+SUM(BASE!$AO$3:$AO$10)/1000,"")</f>
       </c>
       <c r="K3" s="1052">
-        <f>IF(BASE!$B$11=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:K4),"")</f>
+        <f>IF(BASE!$B$11=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:K4)+SUM(BASE!$AO$3:$AO$11)/1000,"")</f>
       </c>
       <c r="L3" s="1052">
-        <f>IF(BASE!$B$12=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:L4),"")</f>
+        <f>IF(BASE!$B$12=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:L4)+SUM(BASE!$AO$3:$AO$12)/1000,"")</f>
       </c>
       <c r="M3" s="1052">
-        <f>IF(BASE!$B$13=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:M4),"")</f>
+        <f>IF(BASE!$B$13=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:M4)+SUM(BASE!$AO$3:$AO$13)/1000,"")</f>
       </c>
       <c r="N3" s="1052">
-        <f>IF(BASE!$B$14=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:N4),"")</f>
+        <f>IF(BASE!$B$14=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:N4)+SUM(BASE!$AO$3:$AO$14)/1000,"")</f>
       </c>
     </row>
     <row r="4" ht="18" thickBot="1">
@@ -27614,40 +27614,40 @@
         <v>99</v>
       </c>
       <c r="C8" s="1052">
-        <f>IF(BASE!$B$15=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:C9),"")</f>
+        <f>IF(BASE!$B$15=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:C9)+SUM(BASE!$AO$3:$AO$15)/1000,"")</f>
       </c>
       <c r="D8" s="1052">
-        <f>IF(BASE!$B$16=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:D9),"")</f>
+        <f>IF(BASE!$B$16=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:D9)+SUM(BASE!$AO$3:$AO$16)/1000,"")</f>
       </c>
       <c r="E8" s="1052">
-        <f>IF(BASE!$B$17=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:E9),"")</f>
+        <f>IF(BASE!$B$17=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:E9)+SUM(BASE!$AO$3:$AO$17)/1000,"")</f>
       </c>
       <c r="F8" s="1052">
-        <f>IF(BASE!$B$18=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:F9),"")</f>
+        <f>IF(BASE!$B$18=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:F9)+SUM(BASE!$AO$3:$AO$18)/1000,"")</f>
       </c>
       <c r="G8" s="1052">
-        <f>IF(BASE!$B$19=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:G9),"")</f>
+        <f>IF(BASE!$B$19=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:G9)+SUM(BASE!$AO$3:$AO$19)/1000,"")</f>
       </c>
       <c r="H8" s="1052">
-        <f>IF(BASE!$B$20=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:H9),"")</f>
+        <f>IF(BASE!$B$20=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:H9)+SUM(BASE!$AO$3:$AO$20)/1000,"")</f>
       </c>
       <c r="I8" s="1052">
-        <f>IF(BASE!$B$21=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:I9),"")</f>
+        <f>IF(BASE!$B$21=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:I9)+SUM(BASE!$AO$3:$AO$21)/1000,"")</f>
       </c>
       <c r="J8" s="1052">
-        <f>IF(BASE!$B$22=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:J9),"")</f>
+        <f>IF(BASE!$B$22=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:J9)+SUM(BASE!$AO$3:$AO$22)/1000,"")</f>
       </c>
       <c r="K8" s="1052">
-        <f>IF(BASE!$B$23=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:K9),"")</f>
+        <f>IF(BASE!$B$23=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:K9)+SUM(BASE!$AO$3:$AO$23)/1000,"")</f>
       </c>
       <c r="L8" s="1052">
-        <f>IF(BASE!$B$24=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:L9),"")</f>
+        <f>IF(BASE!$B$24=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:L9)+SUM(BASE!$AO$3:$AO$24)/1000,"")</f>
       </c>
       <c r="M8" s="1052">
-        <f>IF(BASE!$B$25=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:M9),"")</f>
+        <f>IF(BASE!$B$25=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:M9)+SUM(BASE!$AO$3:$AO$25)/1000,"")</f>
       </c>
       <c r="N8" s="1052">
-        <f>IF(BASE!$B$26=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:N9),"")</f>
+        <f>IF(BASE!$B$26=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:N9)+SUM(BASE!$AO$3:$AO$26)/1000,"")</f>
       </c>
     </row>
     <row r="9" ht="18" thickBot="1">
@@ -27790,40 +27790,40 @@
         <v>100</v>
       </c>
       <c r="C13" s="1052">
-        <f>IF(BASE!$B$27=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:C14),"")</f>
+        <f>IF(BASE!$B$27=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:C14)+SUM(BASE!$AO$3:$AO$27)/1000,"")</f>
       </c>
       <c r="D13" s="1052">
-        <f>IF(BASE!$B$28=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:D14),"")</f>
+        <f>IF(BASE!$B$28=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:D14)+SUM(BASE!$AO$3:$AO$28)/1000,"")</f>
       </c>
       <c r="E13" s="1052">
-        <f>IF(BASE!$B$29=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:E14),"")</f>
+        <f>IF(BASE!$B$29=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:E14)+SUM(BASE!$AO$3:$AO$29)/1000,"")</f>
       </c>
       <c r="F13" s="1052">
-        <f>IF(BASE!$B$30=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:F14),"")</f>
+        <f>IF(BASE!$B$30=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:F14)+SUM(BASE!$AO$3:$AO$30)/1000,"")</f>
       </c>
       <c r="G13" s="1052">
-        <f>IF(BASE!$B$31=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:G14),"")</f>
+        <f>IF(BASE!$B$31=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:G14)+SUM(BASE!$AO$3:$AO$31)/1000,"")</f>
       </c>
       <c r="H13" s="1052">
-        <f>IF(BASE!$B$32=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:H14),"")</f>
+        <f>IF(BASE!$B$32=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:H14)+SUM(BASE!$AO$3:$AO$32)/1000,"")</f>
       </c>
       <c r="I13" s="1052">
-        <f>IF(BASE!$B$33=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:I14),"")</f>
+        <f>IF(BASE!$B$33=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:I14)+SUM(BASE!$AO$3:$AO$33)/1000,"")</f>
       </c>
       <c r="J13" s="1052">
-        <f>IF(BASE!$B$34=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:J14),"")</f>
+        <f>IF(BASE!$B$34=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:J14)+SUM(BASE!$AO$3:$AO$34)/1000,"")</f>
       </c>
       <c r="K13" s="1052">
-        <f>IF(BASE!$B$35=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:K14),"")</f>
+        <f>IF(BASE!$B$35=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:K14)+SUM(BASE!$AO$3:$AO$35)/1000,"")</f>
       </c>
       <c r="L13" s="1052">
-        <f>IF(BASE!$B$36=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:L14),"")</f>
+        <f>IF(BASE!$B$36=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:L14)+SUM(BASE!$AO$3:$AO$36)/1000,"")</f>
       </c>
       <c r="M13" s="1052">
-        <f>IF(BASE!$B$37=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:M14),"")</f>
+        <f>IF(BASE!$B$37=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:M14)+SUM(BASE!$AO$3:$AO$37)/1000,"")</f>
       </c>
       <c r="N13" s="1052">
-        <f>IF(BASE!$B$38=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:N14),"")</f>
+        <f>IF(BASE!$B$38=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:N14)+SUM(BASE!$AO$3:$AO$38)/1000,"")</f>
       </c>
     </row>
     <row r="14" ht="18" thickBot="1">

</xml_diff>

<commit_message>
feat(workbook): caixa final, bloqueado e retiradas nas entradas do fechamento (#110)
- Caixa final (saldo do extrato) informado no fechamento: a diferença para o
  caixa calculado vira ajuste do mês (coluna AO da BASE), somado ao caixa
  acumulado da aba Receita; os meses seguintes partem do caixa informado.
- Bloqueado passa a ser só informado no fechamento (antes: soma atual dos
  limites dos cartões, igual em todos os meses).
- Saldo anterior do caixa inclui dez/(ano-3), que ficava fora do modelo.
- Janela "Entradas do fechamento" com seções de redes sociais, caixa (com o
  valor calculado e o ajuste), sócios/FOPAG (retiradas e saldo do mês, só
  leitura) e parâmetros do ano.
- BASE grava as células de cada linha em ordem de coluna.


Claude-Session: https://claude.ai/code/session_01X7r1acLXPYnBHUwEgBcPmn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v1.xlsx
+++ b/public/workbook_fechamento_v1.xlsx
@@ -27449,40 +27449,40 @@
         <v>98</v>
       </c>
       <c r="C3" s="1052">
-        <f>IF(BASE!$B$3=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:C4),"")</f>
+        <f>IF(BASE!$B$3=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:C4)+SUM(BASE!$AO$3:$AO$3)/1000,"")</f>
       </c>
       <c r="D3" s="1052">
-        <f>IF(BASE!$B$4=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:D4),"")</f>
+        <f>IF(BASE!$B$4=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:D4)+SUM(BASE!$AO$3:$AO$4)/1000,"")</f>
       </c>
       <c r="E3" s="1052">
-        <f>IF(BASE!$B$5=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:E4),"")</f>
+        <f>IF(BASE!$B$5=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:E4)+SUM(BASE!$AO$3:$AO$5)/1000,"")</f>
       </c>
       <c r="F3" s="1052">
-        <f>IF(BASE!$B$6=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:F4),"")</f>
+        <f>IF(BASE!$B$6=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:F4)+SUM(BASE!$AO$3:$AO$6)/1000,"")</f>
       </c>
       <c r="G3" s="1052">
-        <f>IF(BASE!$B$7=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:G4),"")</f>
+        <f>IF(BASE!$B$7=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:G4)+SUM(BASE!$AO$3:$AO$7)/1000,"")</f>
       </c>
       <c r="H3" s="1052">
-        <f>IF(BASE!$B$8=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:H4),"")</f>
+        <f>IF(BASE!$B$8=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:H4)+SUM(BASE!$AO$3:$AO$8)/1000,"")</f>
       </c>
       <c r="I3" s="1052">
-        <f>IF(BASE!$B$9=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:I4),"")</f>
+        <f>IF(BASE!$B$9=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:I4)+SUM(BASE!$AO$3:$AO$9)/1000,"")</f>
       </c>
       <c r="J3" s="1052">
-        <f>IF(BASE!$B$10=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:J4),"")</f>
+        <f>IF(BASE!$B$10=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:J4)+SUM(BASE!$AO$3:$AO$10)/1000,"")</f>
       </c>
       <c r="K3" s="1052">
-        <f>IF(BASE!$B$11=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:K4),"")</f>
+        <f>IF(BASE!$B$11=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:K4)+SUM(BASE!$AO$3:$AO$11)/1000,"")</f>
       </c>
       <c r="L3" s="1052">
-        <f>IF(BASE!$B$12=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:L4),"")</f>
+        <f>IF(BASE!$B$12=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:L4)+SUM(BASE!$AO$3:$AO$12)/1000,"")</f>
       </c>
       <c r="M3" s="1052">
-        <f>IF(BASE!$B$13=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:M4),"")</f>
+        <f>IF(BASE!$B$13=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:M4)+SUM(BASE!$AO$3:$AO$13)/1000,"")</f>
       </c>
       <c r="N3" s="1052">
-        <f>IF(BASE!$B$14=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:N4),"")</f>
+        <f>IF(BASE!$B$14=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:N4)+SUM(BASE!$AO$3:$AO$14)/1000,"")</f>
       </c>
     </row>
     <row r="4" ht="18" thickBot="1">
@@ -27614,40 +27614,40 @@
         <v>99</v>
       </c>
       <c r="C8" s="1052">
-        <f>IF(BASE!$B$15=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:C9),"")</f>
+        <f>IF(BASE!$B$15=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:C9)+SUM(BASE!$AO$3:$AO$15)/1000,"")</f>
       </c>
       <c r="D8" s="1052">
-        <f>IF(BASE!$B$16=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:D9),"")</f>
+        <f>IF(BASE!$B$16=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:D9)+SUM(BASE!$AO$3:$AO$16)/1000,"")</f>
       </c>
       <c r="E8" s="1052">
-        <f>IF(BASE!$B$17=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:E9),"")</f>
+        <f>IF(BASE!$B$17=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:E9)+SUM(BASE!$AO$3:$AO$17)/1000,"")</f>
       </c>
       <c r="F8" s="1052">
-        <f>IF(BASE!$B$18=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:F9),"")</f>
+        <f>IF(BASE!$B$18=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:F9)+SUM(BASE!$AO$3:$AO$18)/1000,"")</f>
       </c>
       <c r="G8" s="1052">
-        <f>IF(BASE!$B$19=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:G9),"")</f>
+        <f>IF(BASE!$B$19=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:G9)+SUM(BASE!$AO$3:$AO$19)/1000,"")</f>
       </c>
       <c r="H8" s="1052">
-        <f>IF(BASE!$B$20=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:H9),"")</f>
+        <f>IF(BASE!$B$20=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:H9)+SUM(BASE!$AO$3:$AO$20)/1000,"")</f>
       </c>
       <c r="I8" s="1052">
-        <f>IF(BASE!$B$21=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:I9),"")</f>
+        <f>IF(BASE!$B$21=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:I9)+SUM(BASE!$AO$3:$AO$21)/1000,"")</f>
       </c>
       <c r="J8" s="1052">
-        <f>IF(BASE!$B$22=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:J9),"")</f>
+        <f>IF(BASE!$B$22=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:J9)+SUM(BASE!$AO$3:$AO$22)/1000,"")</f>
       </c>
       <c r="K8" s="1052">
-        <f>IF(BASE!$B$23=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:K9),"")</f>
+        <f>IF(BASE!$B$23=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:K9)+SUM(BASE!$AO$3:$AO$23)/1000,"")</f>
       </c>
       <c r="L8" s="1052">
-        <f>IF(BASE!$B$24=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:L9),"")</f>
+        <f>IF(BASE!$B$24=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:L9)+SUM(BASE!$AO$3:$AO$24)/1000,"")</f>
       </c>
       <c r="M8" s="1052">
-        <f>IF(BASE!$B$25=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:M9),"")</f>
+        <f>IF(BASE!$B$25=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:M9)+SUM(BASE!$AO$3:$AO$25)/1000,"")</f>
       </c>
       <c r="N8" s="1052">
-        <f>IF(BASE!$B$26=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:N9),"")</f>
+        <f>IF(BASE!$B$26=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:N9)+SUM(BASE!$AO$3:$AO$26)/1000,"")</f>
       </c>
     </row>
     <row r="9" ht="18" thickBot="1">
@@ -27790,40 +27790,40 @@
         <v>100</v>
       </c>
       <c r="C13" s="1052">
-        <f>IF(BASE!$B$27=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:C14),"")</f>
+        <f>IF(BASE!$B$27=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:C14)+SUM(BASE!$AO$3:$AO$27)/1000,"")</f>
       </c>
       <c r="D13" s="1052">
-        <f>IF(BASE!$B$28=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:D14),"")</f>
+        <f>IF(BASE!$B$28=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:D14)+SUM(BASE!$AO$3:$AO$28)/1000,"")</f>
       </c>
       <c r="E13" s="1052">
-        <f>IF(BASE!$B$29=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:E14),"")</f>
+        <f>IF(BASE!$B$29=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:E14)+SUM(BASE!$AO$3:$AO$29)/1000,"")</f>
       </c>
       <c r="F13" s="1052">
-        <f>IF(BASE!$B$30=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:F14),"")</f>
+        <f>IF(BASE!$B$30=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:F14)+SUM(BASE!$AO$3:$AO$30)/1000,"")</f>
       </c>
       <c r="G13" s="1052">
-        <f>IF(BASE!$B$31=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:G14),"")</f>
+        <f>IF(BASE!$B$31=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:G14)+SUM(BASE!$AO$3:$AO$31)/1000,"")</f>
       </c>
       <c r="H13" s="1052">
-        <f>IF(BASE!$B$32=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:H14),"")</f>
+        <f>IF(BASE!$B$32=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:H14)+SUM(BASE!$AO$3:$AO$32)/1000,"")</f>
       </c>
       <c r="I13" s="1052">
-        <f>IF(BASE!$B$33=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:I14),"")</f>
+        <f>IF(BASE!$B$33=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:I14)+SUM(BASE!$AO$3:$AO$33)/1000,"")</f>
       </c>
       <c r="J13" s="1052">
-        <f>IF(BASE!$B$34=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:J14),"")</f>
+        <f>IF(BASE!$B$34=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:J14)+SUM(BASE!$AO$3:$AO$34)/1000,"")</f>
       </c>
       <c r="K13" s="1052">
-        <f>IF(BASE!$B$35=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:K14),"")</f>
+        <f>IF(BASE!$B$35=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:K14)+SUM(BASE!$AO$3:$AO$35)/1000,"")</f>
       </c>
       <c r="L13" s="1052">
-        <f>IF(BASE!$B$36=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:L14),"")</f>
+        <f>IF(BASE!$B$36=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:L14)+SUM(BASE!$AO$3:$AO$36)/1000,"")</f>
       </c>
       <c r="M13" s="1052">
-        <f>IF(BASE!$B$37=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:M14),"")</f>
+        <f>IF(BASE!$B$37=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:M14)+SUM(BASE!$AO$3:$AO$37)/1000,"")</f>
       </c>
       <c r="N13" s="1052">
-        <f>IF(BASE!$B$38=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:N14),"")</f>
+        <f>IF(BASE!$B$38=1,BASE!$AQ$9/1000+SUM(Confronto!$C$4:$N$4,Confronto!$C$9:$N$9,Confronto!$C$14:N14)+SUM(BASE!$AO$3:$AO$38)/1000,"")</f>
       </c>
     </row>
     <row r="14" ht="18" thickBot="1">

</xml_diff>